<commit_message>
updated SQL workbench for both create tables and insert tables
</commit_message>
<xml_diff>
--- a/Springer_Ex3A_tables.xlsx
+++ b/Springer_Ex3A_tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\christopherspringer\Documents\DATA_Labs\W2_Workshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{F9637A4C-C402-4E50-AB05-B50E61C4986F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63A9C969-7CDD-418D-9D3D-844894416620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{2CBDA0D1-2E0B-4F26-A86A-BCDCDFCEA75F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="3" xr2:uid="{2CBDA0D1-2E0B-4F26-A86A-BCDCDFCEA75F}"/>
   </bookViews>
   <sheets>
     <sheet name="Owner" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
   <si>
     <t>owner_id</t>
   </si>
@@ -90,16 +90,48 @@
   </si>
   <si>
     <t>notes</t>
+  </si>
+  <si>
+    <t>Jared Smith</t>
+  </si>
+  <si>
+    <t>555-1111</t>
+  </si>
+  <si>
+    <t>sample_name@email.com</t>
+  </si>
+  <si>
+    <t>Rex</t>
+  </si>
+  <si>
+    <t>Golden Retriever</t>
+  </si>
+  <si>
+    <t>He had a fun time today!</t>
+  </si>
+  <si>
+    <t>Debit</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -134,15 +166,21 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -475,13 +513,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91BBF6F1-9876-4720-96FD-5612DAAB1E00}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -498,18 +536,38 @@
         <v>3</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>1001</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{2A94C1AF-CF00-4173-B06A-AEA6AD9A1B19}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F06B54F8-78BD-43DC-B2D6-94893DFFA57E}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="1"/>
-    <col min="2" max="2" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="6.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="3.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -527,6 +585,23 @@
       </c>
       <c r="E1" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>1001</v>
+      </c>
+      <c r="B2" s="2">
+        <v>1001</v>
+      </c>
+      <c r="C2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -536,11 +611,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECC3AA50-92D9-43AB-B724-9AFBCA89702D}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
     <col min="2" max="2" width="8.88671875" style="2"/>
+    <col min="5" max="5" width="20.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -558,6 +634,23 @@
       </c>
       <c r="E1" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>1001</v>
+      </c>
+      <c r="B2" s="2">
+        <v>1001</v>
+      </c>
+      <c r="C2" s="4">
+        <v>46023</v>
+      </c>
+      <c r="D2" s="5">
+        <v>1.25</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -567,7 +660,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CFD4629-D3E1-442A-AC86-2D801BB558B9}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" style="1" bestFit="1" customWidth="1"/>
@@ -594,6 +687,23 @@
         <v>7</v>
       </c>
     </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>1001</v>
+      </c>
+      <c r="B2" s="2">
+        <v>1001</v>
+      </c>
+      <c r="C2" s="6">
+        <v>25</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="4">
+        <v>46023</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added the values to the tables
</commit_message>
<xml_diff>
--- a/Springer_Ex3A_tables.xlsx
+++ b/Springer_Ex3A_tables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\christopherspringer\Documents\DATA_Labs\W2_Workshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63A9C969-7CDD-418D-9D3D-844894416620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2888CDE-8A65-4BE6-9F9E-D9F22132F35D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="3" xr2:uid="{2CBDA0D1-2E0B-4F26-A86A-BCDCDFCEA75F}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="85">
   <si>
     <t>owner_id</t>
   </si>
@@ -98,9 +98,6 @@
     <t>555-1111</t>
   </si>
   <si>
-    <t>sample_name@email.com</t>
-  </si>
-  <si>
     <t>Rex</t>
   </si>
   <si>
@@ -111,6 +108,195 @@
   </si>
   <si>
     <t>Debit</t>
+  </si>
+  <si>
+    <t>Sarah Johnson</t>
+  </si>
+  <si>
+    <t>555-1112</t>
+  </si>
+  <si>
+    <t>sarah.johnson@email.com</t>
+  </si>
+  <si>
+    <t>Michael Davis</t>
+  </si>
+  <si>
+    <t>555-1113</t>
+  </si>
+  <si>
+    <t>michael.davis@email.com</t>
+  </si>
+  <si>
+    <t>Emily Wilson</t>
+  </si>
+  <si>
+    <t>555-1114</t>
+  </si>
+  <si>
+    <t>emily.wilson@email.com</t>
+  </si>
+  <si>
+    <t>David Brown</t>
+  </si>
+  <si>
+    <t>555-1115</t>
+  </si>
+  <si>
+    <t>david.brown@email.com</t>
+  </si>
+  <si>
+    <t>Jessica Taylor</t>
+  </si>
+  <si>
+    <t>555-1116</t>
+  </si>
+  <si>
+    <t>jessica.taylor@email.com</t>
+  </si>
+  <si>
+    <t>Ryan Martinez</t>
+  </si>
+  <si>
+    <t>555-1117</t>
+  </si>
+  <si>
+    <t>ryan.martinez@email.com</t>
+  </si>
+  <si>
+    <t>Ashley Anderson</t>
+  </si>
+  <si>
+    <t>555-1118</t>
+  </si>
+  <si>
+    <t>ashley.anderson@email.com</t>
+  </si>
+  <si>
+    <t>Matthew Thomas</t>
+  </si>
+  <si>
+    <t>555-1119</t>
+  </si>
+  <si>
+    <t>matthew.thomas@email.com</t>
+  </si>
+  <si>
+    <t>Olivia Harris</t>
+  </si>
+  <si>
+    <t>555-1120</t>
+  </si>
+  <si>
+    <t>olivia.harris@email.com</t>
+  </si>
+  <si>
+    <t>Daniel White</t>
+  </si>
+  <si>
+    <t>555-1121</t>
+  </si>
+  <si>
+    <t>daniel.white@email.com</t>
+  </si>
+  <si>
+    <t>Bella</t>
+  </si>
+  <si>
+    <t>Labrador Retriever</t>
+  </si>
+  <si>
+    <t>Charlie</t>
+  </si>
+  <si>
+    <t>Beagle</t>
+  </si>
+  <si>
+    <t>Luna</t>
+  </si>
+  <si>
+    <t>German Shepherd</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>Poodle</t>
+  </si>
+  <si>
+    <t>Daisy</t>
+  </si>
+  <si>
+    <t>Bulldog</t>
+  </si>
+  <si>
+    <t>Cooper</t>
+  </si>
+  <si>
+    <t>Boxer</t>
+  </si>
+  <si>
+    <t>Molly</t>
+  </si>
+  <si>
+    <t>Dachshund</t>
+  </si>
+  <si>
+    <t>Rocky</t>
+  </si>
+  <si>
+    <t>Siberian Husky</t>
+  </si>
+  <si>
+    <t>Lucy</t>
+  </si>
+  <si>
+    <t>Cocker Spaniel</t>
+  </si>
+  <si>
+    <t>Bailey</t>
+  </si>
+  <si>
+    <t>Border Collie</t>
+  </si>
+  <si>
+    <t>Enjoyed a walk through the neighborhood.</t>
+  </si>
+  <si>
+    <t>Very energetic during the walk.</t>
+  </si>
+  <si>
+    <t>Visited the local dog park.</t>
+  </si>
+  <si>
+    <t>Calm and well-behaved.</t>
+  </si>
+  <si>
+    <t>Played fetch midway through walk.</t>
+  </si>
+  <si>
+    <t>High energy and friendly.</t>
+  </si>
+  <si>
+    <t>Short walk due to weather.</t>
+  </si>
+  <si>
+    <t>Very active and alert.</t>
+  </si>
+  <si>
+    <t>Walked along the river trail.</t>
+  </si>
+  <si>
+    <t>First walk, did very well.</t>
+  </si>
+  <si>
+    <t>Credit</t>
+  </si>
+  <si>
+    <t>Cash</t>
+  </si>
+  <si>
+    <t>jared.smith@email.com</t>
   </si>
 </sst>
 </file>
@@ -118,7 +304,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -170,14 +356,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="46" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -194,6 +383,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -513,13 +706,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91BBF6F1-9876-4720-96FD-5612DAAB1E00}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -547,7 +740,147 @@
         <v>17</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>18</v>
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>1002</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>1003</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>1004</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>1005</v>
+      </c>
+      <c r="B6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>1006</v>
+      </c>
+      <c r="B7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>1007</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>1008</v>
+      </c>
+      <c r="B9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>1009</v>
+      </c>
+      <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>1010</v>
+      </c>
+      <c r="B11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>1011</v>
+      </c>
+      <c r="B12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -560,13 +893,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F06B54F8-78BD-43DC-B2D6-94893DFFA57E}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.21875" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="3.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -595,13 +928,183 @@
         <v>1001</v>
       </c>
       <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
         <v>19</v>
-      </c>
-      <c r="D2" t="s">
-        <v>20</v>
       </c>
       <c r="E2">
         <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>1002</v>
+      </c>
+      <c r="B3" s="2">
+        <v>1002</v>
+      </c>
+      <c r="C3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>1003</v>
+      </c>
+      <c r="B4" s="2">
+        <v>1003</v>
+      </c>
+      <c r="C4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>1004</v>
+      </c>
+      <c r="B5" s="2">
+        <v>1004</v>
+      </c>
+      <c r="C5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" t="s">
+        <v>57</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>1005</v>
+      </c>
+      <c r="B6" s="2">
+        <v>1005</v>
+      </c>
+      <c r="C6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E6">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>1006</v>
+      </c>
+      <c r="B7" s="2">
+        <v>1006</v>
+      </c>
+      <c r="C7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>1007</v>
+      </c>
+      <c r="B8" s="2">
+        <v>1007</v>
+      </c>
+      <c r="C8" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" t="s">
+        <v>63</v>
+      </c>
+      <c r="E8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>1008</v>
+      </c>
+      <c r="B9" s="2">
+        <v>1008</v>
+      </c>
+      <c r="C9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" t="s">
+        <v>65</v>
+      </c>
+      <c r="E9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>1009</v>
+      </c>
+      <c r="B10" s="2">
+        <v>1009</v>
+      </c>
+      <c r="C10" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>1010</v>
+      </c>
+      <c r="B11" s="2">
+        <v>1010</v>
+      </c>
+      <c r="C11" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" t="s">
+        <v>69</v>
+      </c>
+      <c r="E11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>1011</v>
+      </c>
+      <c r="B12" s="2">
+        <v>1011</v>
+      </c>
+      <c r="C12" t="s">
+        <v>70</v>
+      </c>
+      <c r="D12" t="s">
+        <v>71</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -611,12 +1114,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECC3AA50-92D9-43AB-B724-9AFBCA89702D}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="1"/>
-    <col min="2" max="2" width="8.88671875" style="2"/>
-    <col min="5" max="5" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="42.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -646,11 +1151,181 @@
       <c r="C2" s="4">
         <v>46023</v>
       </c>
-      <c r="D2" s="5">
-        <v>1.25</v>
-      </c>
-      <c r="E2" t="s">
-        <v>21</v>
+      <c r="D2" s="7">
+        <v>30</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>1002</v>
+      </c>
+      <c r="B3" s="2">
+        <v>1002</v>
+      </c>
+      <c r="C3" s="4">
+        <v>46024</v>
+      </c>
+      <c r="D3" s="7">
+        <v>45</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>1003</v>
+      </c>
+      <c r="B4" s="2">
+        <v>1003</v>
+      </c>
+      <c r="C4" s="4">
+        <v>46025</v>
+      </c>
+      <c r="D4" s="7">
+        <v>30</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>1004</v>
+      </c>
+      <c r="B5" s="2">
+        <v>1004</v>
+      </c>
+      <c r="C5" s="4">
+        <v>46026</v>
+      </c>
+      <c r="D5" s="7">
+        <v>60</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>1005</v>
+      </c>
+      <c r="B6" s="2">
+        <v>1005</v>
+      </c>
+      <c r="C6" s="4">
+        <v>46027</v>
+      </c>
+      <c r="D6" s="7">
+        <v>35</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>1006</v>
+      </c>
+      <c r="B7" s="2">
+        <v>1006</v>
+      </c>
+      <c r="C7" s="4">
+        <v>46028</v>
+      </c>
+      <c r="D7" s="7">
+        <v>40</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>1007</v>
+      </c>
+      <c r="B8" s="2">
+        <v>1007</v>
+      </c>
+      <c r="C8" s="4">
+        <v>46029</v>
+      </c>
+      <c r="D8" s="7">
+        <v>50</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>1008</v>
+      </c>
+      <c r="B9" s="2">
+        <v>1008</v>
+      </c>
+      <c r="C9" s="4">
+        <v>46030</v>
+      </c>
+      <c r="D9" s="7">
+        <v>25</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>1009</v>
+      </c>
+      <c r="B10" s="2">
+        <v>1009</v>
+      </c>
+      <c r="C10" s="4">
+        <v>46031</v>
+      </c>
+      <c r="D10" s="7">
+        <v>65</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>1010</v>
+      </c>
+      <c r="B11" s="2">
+        <v>1010</v>
+      </c>
+      <c r="C11" s="4">
+        <v>46032</v>
+      </c>
+      <c r="D11" s="7">
+        <v>45</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>1011</v>
+      </c>
+      <c r="B12" s="2">
+        <v>1011</v>
+      </c>
+      <c r="C12" s="4">
+        <v>46033</v>
+      </c>
+      <c r="D12" s="7">
+        <v>30</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -660,14 +1335,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CFD4629-D3E1-442A-AC86-2D801BB558B9}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.21875" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -694,14 +1369,184 @@
       <c r="B2" s="2">
         <v>1001</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="5">
         <v>25</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E2" s="4">
         <v>46023</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>1002</v>
+      </c>
+      <c r="B3" s="2">
+        <v>1002</v>
+      </c>
+      <c r="C3" s="5">
+        <v>30</v>
+      </c>
+      <c r="D3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E3" s="4">
+        <v>46024</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>1003</v>
+      </c>
+      <c r="B4" s="2">
+        <v>1003</v>
+      </c>
+      <c r="C4" s="5">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="4">
+        <v>46025</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>1004</v>
+      </c>
+      <c r="B5" s="2">
+        <v>1004</v>
+      </c>
+      <c r="C5" s="5">
+        <v>35</v>
+      </c>
+      <c r="D5" t="s">
+        <v>83</v>
+      </c>
+      <c r="E5" s="4">
+        <v>46026</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>1005</v>
+      </c>
+      <c r="B6" s="2">
+        <v>1005</v>
+      </c>
+      <c r="C6" s="5">
+        <v>25</v>
+      </c>
+      <c r="D6" t="s">
+        <v>82</v>
+      </c>
+      <c r="E6" s="4">
+        <v>46027</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>1006</v>
+      </c>
+      <c r="B7" s="2">
+        <v>1006</v>
+      </c>
+      <c r="C7" s="5">
+        <v>30</v>
+      </c>
+      <c r="D7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="4">
+        <v>46028</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>1007</v>
+      </c>
+      <c r="B8" s="2">
+        <v>1007</v>
+      </c>
+      <c r="C8" s="5">
+        <v>40</v>
+      </c>
+      <c r="D8" t="s">
+        <v>82</v>
+      </c>
+      <c r="E8" s="4">
+        <v>46029</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>1008</v>
+      </c>
+      <c r="B9" s="2">
+        <v>1008</v>
+      </c>
+      <c r="C9" s="5">
+        <v>20</v>
+      </c>
+      <c r="D9" t="s">
+        <v>83</v>
+      </c>
+      <c r="E9" s="4">
+        <v>46030</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>1009</v>
+      </c>
+      <c r="B10" s="2">
+        <v>1009</v>
+      </c>
+      <c r="C10" s="5">
+        <v>35</v>
+      </c>
+      <c r="D10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" s="4">
+        <v>46031</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>1010</v>
+      </c>
+      <c r="B11" s="2">
+        <v>1010</v>
+      </c>
+      <c r="C11" s="5">
+        <v>30</v>
+      </c>
+      <c r="D11" t="s">
+        <v>82</v>
+      </c>
+      <c r="E11" s="4">
+        <v>46032</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>1011</v>
+      </c>
+      <c r="B12" s="2">
+        <v>1011</v>
+      </c>
+      <c r="C12" s="5">
+        <v>25</v>
+      </c>
+      <c r="D12" t="s">
+        <v>83</v>
+      </c>
+      <c r="E12" s="4">
+        <v>46033</v>
       </c>
     </row>
   </sheetData>

</xml_diff>